<commit_message>
Últimos cambios en tablas y figuras finales
</commit_message>
<xml_diff>
--- a/Output/Tables/desc_cluster.xlsx
+++ b/Output/Tables/desc_cluster.xlsx
@@ -340,7 +340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -735,27 +735,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   717 (100%)   </t>
+          <t xml:space="preserve">  458 (63.9%)   </t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">     420 (100%)     </t>
+          <t xml:space="preserve">    330 (78.6%)     </t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    734 (100%)     </t>
+          <t xml:space="preserve">    616 (83.9%)    </t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">             350 (100%)             </t>
+          <t xml:space="preserve">            258 (73.7%)             </t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .    </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
@@ -767,27 +767,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   717 (100%)   </t>
+          <t xml:space="preserve">   50 (6.97%)   </t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">     420 (100%)     </t>
+          <t xml:space="preserve">     20 (4.76%)     </t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">    734 (100%)     </t>
+          <t xml:space="preserve">    52 (7.08%)     </t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">             350 (100%)             </t>
+          <t xml:space="preserve">             64 (18.3%)             </t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .    </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
@@ -1370,91 +1370,91 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>incontinence_cat, N (%): 'Missing'</t>
+          <t>incontinence_cat, N (%):</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">   717 (100%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">     420 (100%)     </t>
+          <t xml:space="preserve">                    </t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    734 (100%)     </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">             350 (100%)             </t>
+          <t xml:space="preserve">                                    </t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .    </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>social_risk, N (%):</t>
+          <t xml:space="preserve">    Fecal and urinary</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   1 (0.14%)    </t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    </t>
+          <t xml:space="preserve">     9 (2.14%)      </t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">     7 (0.95%)     </t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                    </t>
+          <t xml:space="preserve">            224 (64.0%)             </t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    No</t>
+          <t xml:space="preserve">    Fecal</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  364 (50.8%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    247 (58.8%)     </t>
+          <t xml:space="preserve">     2 (0.48%)      </t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    459 (62.5%)    </t>
+          <t xml:space="preserve">     6 (0.82%)     </t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            223 (63.7%)             </t>
+          <t xml:space="preserve">             0 (0.00%)              </t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1466,27 +1466,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Yes</t>
+          <t xml:space="preserve">    Urinary</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">   43 (6.00%)   </t>
+          <t xml:space="preserve">  175 (24.4%)   </t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">    124 (29.5%)     </t>
+          <t xml:space="preserve">    181 (43.1%)     </t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">    50 (6.81%)     </t>
+          <t xml:space="preserve">    508 (69.2%)    </t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">             35 (10.0%)             </t>
+          <t xml:space="preserve">            111 (31.7%)             </t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1498,27 +1498,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    None/None registered</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  310 (43.2%)   </t>
+          <t xml:space="preserve">  541 (75.5%)   </t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">     49 (11.7%)     </t>
+          <t xml:space="preserve">    228 (54.3%)     </t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    225 (30.7%)    </t>
+          <t xml:space="preserve">    213 (29.0%)    </t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">             92 (26.3%)             </t>
+          <t xml:space="preserve">             15 (4.29%)             </t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1530,7 +1530,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TIRS_cat, N (%):</t>
+          <t>social_risk, N (%):</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1562,27 +1562,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    si</t>
+          <t xml:space="preserve">    No</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  155 (21.6%)   </t>
+          <t xml:space="preserve">  364 (50.8%)   </t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    335 (79.8%)     </t>
+          <t xml:space="preserve">    247 (58.8%)     </t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    147 (20.0%)    </t>
+          <t xml:space="preserve">    459 (62.5%)    </t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">             69 (19.7%)             </t>
+          <t xml:space="preserve">            223 (63.7%)             </t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1594,27 +1594,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    Yes</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">   61 (8.51%)   </t>
+          <t xml:space="preserve">   43 (6.00%)   </t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">     6 (1.43%)      </t>
+          <t xml:space="preserve">    124 (29.5%)     </t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">     1 (0.14%)     </t>
+          <t xml:space="preserve">    50 (6.81%)     </t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">             0 (0.00%)              </t>
+          <t xml:space="preserve">             35 (10.0%)             </t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1626,39 +1626,39 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TIRS_num, Median [25th;75th]</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0.00 [0.00;0.00]</t>
+          <t xml:space="preserve">  310 (43.2%)   </t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1.00 [1.00;2.00]  </t>
+          <t xml:space="preserve">     49 (11.7%)     </t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.00 [0.00;0.00]  </t>
+          <t xml:space="preserve">    225 (30.7%)    </t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">          0.00 [0.00;0.00]          </t>
+          <t xml:space="preserve">             92 (26.3%)             </t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>living_alone, N (%):</t>
+          <t>TIRS_cat, N (%):</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1690,27 +1690,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    No</t>
+          <t xml:space="preserve">    si</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  689 (96.1%)   </t>
+          <t xml:space="preserve">  155 (21.6%)   </t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">     90 (21.4%)     </t>
+          <t xml:space="preserve">    335 (79.8%)     </t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    696 (94.8%)    </t>
+          <t xml:space="preserve">    147 (20.0%)    </t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">            318 (90.9%)             </t>
+          <t xml:space="preserve">             69 (19.7%)             </t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1722,27 +1722,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Yes</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">   28 (3.91%)   </t>
+          <t xml:space="preserve">   61 (8.51%)   </t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    330 (78.6%)     </t>
+          <t xml:space="preserve">     6 (1.43%)      </t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    38 (5.18%)     </t>
+          <t xml:space="preserve">     1 (0.14%)     </t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">             32 (9.14%)             </t>
+          <t xml:space="preserve">             0 (0.00%)              </t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1754,27 +1754,27 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>need_household_adapt, N (%):</t>
+          <t>TIRS_num, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t>0.00 [0.00;0.00]</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    </t>
+          <t xml:space="preserve">  1.00 [1.00;2.00]  </t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve"> 0.00 [0.00;0.00]  </t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                    </t>
+          <t xml:space="preserve">          0.00 [0.00;0.00]          </t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1786,32 +1786,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Yes</t>
+          <t>living_alone, N (%):</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  164 (22.9%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">    185 (44.0%)     </t>
+          <t xml:space="preserve">                    </t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">    170 (23.2%)    </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">             71 (20.3%)             </t>
+          <t xml:space="preserve">                                    </t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
@@ -1823,22 +1823,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">  553 (77.1%)   </t>
+          <t xml:space="preserve">  689 (96.1%)   </t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">    235 (56.0%)     </t>
+          <t xml:space="preserve">     90 (21.4%)     </t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">    564 (76.8%)    </t>
+          <t xml:space="preserve">    696 (94.8%)    </t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">            279 (79.7%)             </t>
+          <t xml:space="preserve">            318 (90.9%)             </t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -1850,91 +1850,91 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Single_PHC, N (%):</t>
+          <t xml:space="preserve">    Yes</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   28 (3.91%)   </t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    </t>
+          <t xml:space="preserve">    330 (78.6%)     </t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    38 (5.18%)     </t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                    </t>
+          <t xml:space="preserve">             32 (9.14%)             </t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Equip_Atdom</t>
+          <t>need_household_adapt, N (%):</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">  210 (29.3%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">    194 (46.2%)     </t>
+          <t xml:space="preserve">                    </t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">    260 (35.4%)    </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">            116 (33.1%)             </t>
+          <t xml:space="preserve">                                    </t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Equip_Inf</t>
+          <t xml:space="preserve">    Yes</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">   94 (13.1%)   </t>
+          <t xml:space="preserve">  164 (22.9%)   </t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">     63 (15.0%)     </t>
+          <t xml:space="preserve">    185 (44.0%)     </t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">    103 (14.0%)    </t>
+          <t xml:space="preserve">    170 (23.2%)    </t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">             52 (14.9%)             </t>
+          <t xml:space="preserve">             71 (20.3%)             </t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -1946,27 +1946,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">    UAB_consulta</t>
+          <t xml:space="preserve">    No</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">  413 (57.6%)   </t>
+          <t xml:space="preserve">  553 (77.1%)   </t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">    163 (38.8%)     </t>
+          <t xml:space="preserve">    235 (56.0%)     </t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">    371 (50.5%)    </t>
+          <t xml:space="preserve">    564 (76.8%)    </t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">            182 (52.0%)             </t>
+          <t xml:space="preserve">            279 (79.7%)             </t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -1978,7 +1978,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Home_based_PHC_org, N (%):</t>
+          <t>Single_PHC, N (%):</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2079,22 +2079,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  157 (21.9%)   </t>
+          <t xml:space="preserve">  413 (57.6%)   </t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">     52 (12.4%)     </t>
+          <t xml:space="preserve">    163 (38.8%)     </t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    134 (18.3%)    </t>
+          <t xml:space="preserve">    371 (50.5%)    </t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">             67 (19.1%)             </t>
+          <t xml:space="preserve">            182 (52.0%)             </t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2106,91 +2106,91 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    UAB_consulta_reforc</t>
+          <t>Home_based_PHC_org, N (%):</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  256 (35.7%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    111 (26.4%)     </t>
+          <t xml:space="preserve">                    </t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    237 (32.3%)    </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            115 (32.9%)             </t>
+          <t xml:space="preserve">                                    </t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PHC_name, N (%):</t>
+          <t xml:space="preserve">    Equip_Atdom</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  210 (29.3%)   </t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    </t>
+          <t xml:space="preserve">    194 (46.2%)     </t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    260 (35.4%)    </t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                    </t>
+          <t xml:space="preserve">            116 (33.1%)             </t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Borrell</t>
+          <t xml:space="preserve">    Equip_Inf</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  123 (17.2%)   </t>
+          <t xml:space="preserve">   94 (13.1%)   </t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    132 (31.4%)     </t>
+          <t xml:space="preserve">     63 (15.0%)     </t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    132 (18.0%)    </t>
+          <t xml:space="preserve">    103 (14.0%)    </t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">             53 (15.1%)             </t>
+          <t xml:space="preserve">             52 (14.9%)             </t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2202,27 +2202,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Casanova</t>
+          <t xml:space="preserve">    UAB_consulta</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">   94 (13.1%)   </t>
+          <t xml:space="preserve">  157 (21.9%)   </t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">     63 (15.0%)     </t>
+          <t xml:space="preserve">     52 (12.4%)     </t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">    103 (14.0%)    </t>
+          <t xml:space="preserve">    134 (18.3%)    </t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">             52 (14.9%)             </t>
+          <t xml:space="preserve">             67 (19.1%)             </t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2234,27 +2234,27 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Montnegre_1</t>
+          <t xml:space="preserve">    UAB_consulta_reforc</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">   83 (11.6%)   </t>
+          <t xml:space="preserve">  256 (35.7%)   </t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">     29 (6.90%)     </t>
+          <t xml:space="preserve">    111 (26.4%)     </t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">    78 (10.6%)     </t>
+          <t xml:space="preserve">    237 (32.3%)    </t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">             33 (9.43%)             </t>
+          <t xml:space="preserve">            115 (32.9%)             </t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2266,39 +2266,39 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Montnegre_2</t>
+          <t>PHC_name, N (%):</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">   74 (10.3%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">     23 (5.48%)     </t>
+          <t xml:space="preserve">                    </t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">    56 (7.63%)     </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">             34 (9.71%)             </t>
+          <t xml:space="preserve">                                    </t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Marc_Aureli</t>
+          <t xml:space="preserve">    Borrell</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2308,17 +2308,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">     52 (12.4%)     </t>
+          <t xml:space="preserve">    132 (31.4%)     </t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">    100 (13.6%)    </t>
+          <t xml:space="preserve">    132 (18.0%)    </t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">             56 (16.0%)             </t>
+          <t xml:space="preserve">             53 (15.1%)             </t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2330,27 +2330,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Sant_Elies</t>
+          <t xml:space="preserve">    Casanova</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">  133 (18.5%)   </t>
+          <t xml:space="preserve">   94 (13.1%)   </t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">     59 (14.0%)     </t>
+          <t xml:space="preserve">     63 (15.0%)     </t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">    137 (18.7%)    </t>
+          <t xml:space="preserve">    103 (14.0%)    </t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">             59 (16.9%)             </t>
+          <t xml:space="preserve">             52 (14.9%)             </t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2362,27 +2362,27 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Lluch</t>
+          <t xml:space="preserve">    Montnegre_1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   87 (12.1%)   </t>
+          <t xml:space="preserve">   83 (11.6%)   </t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">     62 (14.8%)     </t>
+          <t xml:space="preserve">     29 (6.90%)     </t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">    128 (17.4%)    </t>
+          <t xml:space="preserve">    78 (10.6%)     </t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">             63 (18.0%)             </t>
+          <t xml:space="preserve">             33 (9.43%)             </t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2394,155 +2394,155 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>heart_failure, N (%): si</t>
+          <t xml:space="preserve">    Montnegre_2</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">   28 (3.91%)   </t>
+          <t xml:space="preserve">   74 (10.3%)   </t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">     90 (21.4%)     </t>
+          <t xml:space="preserve">     23 (5.48%)     </t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">    289 (39.4%)    </t>
+          <t xml:space="preserve">    56 (7.63%)     </t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">             55 (15.7%)             </t>
+          <t xml:space="preserve">             34 (9.71%)             </t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ischemic_heart, N (%): si</t>
+          <t xml:space="preserve">    Marc_Aureli</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">   13 (1.81%)   </t>
+          <t xml:space="preserve">  123 (17.2%)   </t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">     30 (7.14%)     </t>
+          <t xml:space="preserve">     52 (12.4%)     </t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">    169 (23.0%)    </t>
+          <t xml:space="preserve">    100 (13.6%)    </t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">             21 (6.00%)             </t>
+          <t xml:space="preserve">             56 (16.0%)             </t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>arrhythmias, N (%): si</t>
+          <t xml:space="preserve">    Sant_Elies</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  120 (16.7%)   </t>
+          <t xml:space="preserve">  133 (18.5%)   </t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">    116 (27.6%)     </t>
+          <t xml:space="preserve">     59 (14.0%)     </t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">    296 (40.3%)    </t>
+          <t xml:space="preserve">    137 (18.7%)    </t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">             93 (26.6%)             </t>
+          <t xml:space="preserve">             59 (16.9%)             </t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>dementia, N (%): si</t>
+          <t xml:space="preserve">    Lluch</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">   45 (6.28%)   </t>
+          <t xml:space="preserve">   87 (12.1%)   </t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">     38 (9.05%)     </t>
+          <t xml:space="preserve">     62 (14.8%)     </t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">    82 (11.2%)     </t>
+          <t xml:space="preserve">    128 (17.4%)    </t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">            229 (65.4%)             </t>
+          <t xml:space="preserve">             63 (18.0%)             </t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>parkinson, N (%): si</t>
+          <t>heart_failure, N (%): si</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   12 (1.67%)   </t>
+          <t xml:space="preserve">   28 (3.91%)   </t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">     10 (2.38%)     </t>
+          <t xml:space="preserve">     90 (21.4%)     </t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">    94 (12.8%)     </t>
+          <t xml:space="preserve">    289 (39.4%)    </t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">             41 (11.7%)             </t>
+          <t xml:space="preserve">             55 (15.7%)             </t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -2554,12 +2554,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>stroke, N (%): si</t>
+          <t>ischemic_heart, N (%): si</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">   36 (5.02%)   </t>
+          <t xml:space="preserve">   13 (1.81%)   </t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2569,12 +2569,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">    206 (28.1%)    </t>
+          <t xml:space="preserve">    169 (23.0%)    </t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">             80 (22.9%)             </t>
+          <t xml:space="preserve">             21 (6.00%)             </t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -2586,27 +2586,27 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>diabetes, N (%): si</t>
+          <t>arrhythmias, N (%): si</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">   38 (5.30%)   </t>
+          <t xml:space="preserve">  120 (16.7%)   </t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">     92 (21.9%)     </t>
+          <t xml:space="preserve">    116 (27.6%)     </t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">    241 (32.8%)    </t>
+          <t xml:space="preserve">    296 (40.3%)    </t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">             79 (22.6%)             </t>
+          <t xml:space="preserve">             93 (26.6%)             </t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2618,27 +2618,27 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>hyperlipidemia, N (%): si</t>
+          <t>dementia, N (%): si</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">   40 (5.58%)   </t>
+          <t xml:space="preserve">   45 (6.28%)   </t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">     61 (14.5%)     </t>
+          <t xml:space="preserve">     38 (9.05%)     </t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">    117 (15.9%)    </t>
+          <t xml:space="preserve">    82 (11.2%)     </t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">             53 (15.1%)             </t>
+          <t xml:space="preserve">            229 (65.4%)             </t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2650,27 +2650,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ckd, N (%): si</t>
+          <t>parkinson, N (%): si</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">   56 (7.81%)   </t>
+          <t xml:space="preserve">   12 (1.67%)   </t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">    107 (25.5%)     </t>
+          <t xml:space="preserve">     10 (2.38%)     </t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">    406 (55.3%)    </t>
+          <t xml:space="preserve">    94 (12.8%)     </t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">             95 (27.1%)             </t>
+          <t xml:space="preserve">             41 (11.7%)             </t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -2682,27 +2682,27 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>copd, N (%): si</t>
+          <t>stroke, N (%): si</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">   60 (8.37%)   </t>
+          <t xml:space="preserve">   36 (5.02%)   </t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">     87 (20.7%)     </t>
+          <t xml:space="preserve">     30 (7.14%)     </t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">    170 (23.2%)    </t>
+          <t xml:space="preserve">    206 (28.1%)    </t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">             34 (9.71%)             </t>
+          <t xml:space="preserve">             80 (22.9%)             </t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -2714,59 +2714,59 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>respiratory_failure, N (%): si</t>
+          <t>diabetes, N (%): si</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">   10 (1.39%)   </t>
+          <t xml:space="preserve">   38 (5.30%)   </t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">     11 (2.62%)     </t>
+          <t xml:space="preserve">     92 (21.9%)     </t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">    26 (3.54%)     </t>
+          <t xml:space="preserve">    241 (32.8%)    </t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">             7 (2.00%)              </t>
+          <t xml:space="preserve">             79 (22.6%)             </t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.060  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Arthritis_osteoarthritis, N (%): si</t>
+          <t>hyperlipidemia, N (%): si</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">  130 (18.1%)   </t>
+          <t xml:space="preserve">   40 (5.58%)   </t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">    235 (56.0%)     </t>
+          <t xml:space="preserve">     61 (14.5%)     </t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">    530 (72.2%)    </t>
+          <t xml:space="preserve">    117 (15.9%)    </t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">            162 (46.3%)             </t>
+          <t xml:space="preserve">             53 (15.1%)             </t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -2778,59 +2778,59 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>hip_fracture, N (%): si</t>
+          <t>ckd, N (%): si</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.42%)    </t>
+          <t xml:space="preserve">   56 (7.81%)   </t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">     6 (1.43%)      </t>
+          <t xml:space="preserve">    107 (25.5%)     </t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">     7 (0.95%)     </t>
+          <t xml:space="preserve">    406 (55.3%)    </t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">             5 (1.43%)              </t>
+          <t xml:space="preserve">             95 (27.1%)             </t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.269  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>osteoporosis, N (%): si</t>
+          <t>copd, N (%): si</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">  107 (14.9%)   </t>
+          <t xml:space="preserve">   60 (8.37%)   </t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">    122 (29.0%)     </t>
+          <t xml:space="preserve">     87 (20.7%)     </t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t xml:space="preserve">    193 (26.3%)    </t>
+          <t xml:space="preserve">    170 (23.2%)    </t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">             95 (27.1%)             </t>
+          <t xml:space="preserve">             34 (9.71%)             </t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -2842,59 +2842,59 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>anxiety_depression, N (%): si</t>
+          <t>respiratory_failure, N (%): si</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">  111 (15.5%)   </t>
+          <t xml:space="preserve">   10 (1.39%)   </t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">    174 (41.4%)     </t>
+          <t xml:space="preserve">     11 (2.62%)     </t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t xml:space="preserve">    452 (61.6%)    </t>
+          <t xml:space="preserve">    26 (3.54%)     </t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">            154 (44.0%)             </t>
+          <t xml:space="preserve">             7 (2.00%)              </t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.060  </t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>anemia, N (%): si</t>
+          <t>Arthritis_osteoarthritis, N (%): si</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">   38 (5.30%)   </t>
+          <t xml:space="preserve">  130 (18.1%)   </t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">     45 (10.7%)     </t>
+          <t xml:space="preserve">    235 (56.0%)     </t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t xml:space="preserve">    87 (11.9%)     </t>
+          <t xml:space="preserve">    530 (72.2%)    </t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">             49 (14.0%)             </t>
+          <t xml:space="preserve">            162 (46.3%)             </t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -2906,59 +2906,59 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>uti, N (%): si</t>
+          <t>hip_fracture, N (%): si</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">   62 (8.65%)   </t>
+          <t xml:space="preserve">   3 (0.42%)    </t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">     75 (17.9%)     </t>
+          <t xml:space="preserve">     6 (1.43%)      </t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t xml:space="preserve">    166 (22.6%)    </t>
+          <t xml:space="preserve">     7 (0.95%)     </t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">            128 (36.6%)             </t>
+          <t xml:space="preserve">             5 (1.43%)              </t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.238  </t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>glaucoma, N (%): si</t>
+          <t>osteoporosis, N (%): si</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">   70 (9.76%)   </t>
+          <t xml:space="preserve">  107 (14.9%)   </t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">     65 (15.5%)     </t>
+          <t xml:space="preserve">    122 (29.0%)     </t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t xml:space="preserve">    128 (17.4%)    </t>
+          <t xml:space="preserve">    193 (26.3%)    </t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">             38 (10.9%)             </t>
+          <t xml:space="preserve">             95 (27.1%)             </t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -2970,27 +2970,27 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Cancer, N (%): si</t>
+          <t>anxiety_depression, N (%): si</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (1.12%)    </t>
+          <t xml:space="preserve">  111 (15.5%)   </t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">     35 (8.33%)     </t>
+          <t xml:space="preserve">    174 (41.4%)     </t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t xml:space="preserve">    39 (5.31%)     </t>
+          <t xml:space="preserve">    452 (61.6%)    </t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">             17 (4.86%)             </t>
+          <t xml:space="preserve">            154 (44.0%)             </t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3002,32 +3002,160 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>anemia, N (%): si</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   38 (5.30%)   </t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     45 (10.7%)     </t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    87 (11.9%)     </t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             49 (14.0%)             </t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> &lt;0.001  </t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>uti, N (%): si</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   62 (8.65%)   </t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     75 (17.9%)     </t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    166 (22.6%)    </t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            128 (36.6%)             </t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> &lt;0.001  </t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>glaucoma, N (%): si</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   70 (9.76%)   </t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     65 (15.5%)     </t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    128 (17.4%)    </t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             38 (10.9%)             </t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> &lt;0.001  </t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Cancer, N (%): si</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   8 (1.12%)    </t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     35 (8.33%)     </t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    39 (5.31%)     </t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             17 (4.86%)             </t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> &lt;0.001  </t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>Liver_disease, N (%): si</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t xml:space="preserve">   1 (0.14%)    </t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t xml:space="preserve">     1 (0.24%)      </t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t xml:space="preserve">     6 (0.82%)     </t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t xml:space="preserve">             1 (0.29%)              </t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.226  </t>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  0.202  </t>
         </is>
       </c>
     </row>

</xml_diff>